<commit_message>
ISO W10 sapuan FAT: FAT-FRM-02 (putaran 2), FAT-FRM-01
Lolos gerbang mesin W10 dan pemeriksa bahasa buta (semua skor >= 4).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BhkCQM7h3krZb9kjY2Nate
</commit_message>
<xml_diff>
--- a/out/03_FAT/SNX-FAT-FRM-02 Financial Information Access Authorization Records (Rev00 DRAFT).xlsx
+++ b/out/03_FAT/SNX-FAT-FRM-02 Financial Information Access Authorization Records (Rev00 DRAFT).xlsx
@@ -7,7 +7,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worksheet" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform Access" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Platform Access'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -171,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -238,6 +241,21 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -512,7 +530,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -538,9 +556,15 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4" ht="15" customHeight="1" s="12">
-      <c r="A4" s="15" t="inlineStr">
+    <row r="3" s="12">
+      <c r="A3" s="23" t="n"/>
+      <c r="B3" s="23" t="n"/>
+      <c r="C3" s="23" t="n"/>
+      <c r="D3" s="23" t="n"/>
+      <c r="E3" s="23" t="n"/>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" s="12">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Nomor dokumen</t>
         </is>
@@ -550,9 +574,12 @@
           <t>SNX-FAT-FRM-02</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="12">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="C4" s="23" t="n"/>
+      <c r="D4" s="23" t="n"/>
+      <c r="E4" s="23" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="12">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
@@ -562,9 +589,12 @@
           <t>Financial Information Access Authorization Records</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="12">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="C5" s="23" t="n"/>
+      <c r="D5" s="23" t="n"/>
+      <c r="E5" s="23" t="n"/>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="12">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Revisi</t>
         </is>
@@ -574,9 +604,12 @@
           <t>00 (DRAFT)</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="12">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="C6" s="23" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="23" t="n"/>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="12">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Tanggal draft</t>
         </is>
@@ -586,9 +619,12 @@
           <t>15 Oktober 2026</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="12">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="C7" s="23" t="n"/>
+      <c r="D7" s="23" t="n"/>
+      <c r="E7" s="23" t="n"/>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="12">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Tanggal efektif</t>
         </is>
@@ -598,9 +634,12 @@
           <t>Ditetapkan saat pengesahan</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="12">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="23" t="n"/>
+      <c r="E8" s="23" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="12">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Klasifikasi</t>
         </is>
@@ -610,9 +649,12 @@
           <t>RESTRICTED (Internal)</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="12">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="C9" s="23" t="n"/>
+      <c r="D9" s="23" t="n"/>
+      <c r="E9" s="23" t="n"/>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="12">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Pemilik dokumen</t>
         </is>
@@ -622,9 +664,12 @@
           <t>Finance Lead</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="12">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="C10" s="23" t="n"/>
+      <c r="D10" s="23" t="n"/>
+      <c r="E10" s="23" t="n"/>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="12">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>Disetujui oleh</t>
         </is>
@@ -634,9 +679,12 @@
           <t>Samuel Kristanto Utomo / President Director</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="C11" s="23" t="n"/>
+      <c r="D11" s="23" t="n"/>
+      <c r="E11" s="23" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" s="12">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>Acuan ISO 9001:2015</t>
         </is>
@@ -646,9 +694,12 @@
           <t>Klausul 7.5.3 (USULAN, perlu konfirmasi konsultan)</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="12">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="C12" s="23" t="n"/>
+      <c r="D12" s="23" t="n"/>
+      <c r="E12" s="23" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="12">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Acuan ISO/IEC 27001:2022</t>
         </is>
@@ -658,9 +709,12 @@
           <t>Kontrol Annex A 5.3, 5.15, 5.18, 8.3 (USULAN, perlu konfirmasi konsultan)</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="12">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
+      <c r="E13" s="23" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1" s="12">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Masa simpan record</t>
         </is>
@@ -670,9 +724,12 @@
           <t>Berlaku sampai digantikan; versi lama minimal 10 tahun (USULAN)</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="23.85" customHeight="1" s="12">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="C14" s="23" t="n"/>
+      <c r="D14" s="23" t="n"/>
+      <c r="E14" s="23" t="n"/>
+    </row>
+    <row r="15" ht="43.5" customHeight="1" s="12">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Tujuan</t>
         </is>
@@ -682,59 +739,79 @@
           <t>Mencatat akses ke data dan informasi departemen Finance (dokumen keuangan, platform pajak dan bank) beserta pemegang aksesnya.</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="C15" s="23" t="n"/>
+      <c r="D15" s="23" t="n"/>
+      <c r="E15" s="23" t="n"/>
+    </row>
+    <row r="16" ht="43.5" customHeight="1" s="12">
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>Finance Lead: peran pemeriksa dan penyetuju FAT; jabatannya belum terisi, dan sampai terisi peran ini dijalankan Direktur (USULAN).</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="12">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="C16" s="23" t="n"/>
+      <c r="D16" s="23" t="n"/>
+      <c r="E16" s="23" t="n"/>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="12">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Cara pakai</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="12">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="B17" s="23" t="n"/>
+      <c r="C17" s="23" t="n"/>
+      <c r="D17" s="23" t="n"/>
+      <c r="E17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="12">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Finance Staff mengisi sheet Worksheet, satu baris per dokumen (USULAN).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="12">
-      <c r="A19" s="18" t="inlineStr">
+          <t>Finance Staff mengisi sheet Worksheet dengan satu baris untuk setiap dokumen (USULAN).</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n"/>
+      <c r="D18" s="23" t="n"/>
+      <c r="E18" s="23" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1" s="12">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>Finance Staff mengisi sheet Platform Access, satu baris per platform (USULAN).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="23.85" customHeight="1" s="12">
-      <c r="A20" s="18" t="inlineStr">
+          <t>Isi sheet Platform Access dengan satu baris untuk setiap platform (USULAN).</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n"/>
+      <c r="D19" s="23" t="n"/>
+      <c r="E19" s="23" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1" s="12">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>Finance Staff menulis pemegang akses sebagai kelompok atau sebagai nama dan jabatan, tanpa kata sandi, PIN, atau token (USULAN).</t>
-        </is>
-      </c>
+          <t>Tulis pemegang akses sebagai kelompok atau sebagai nama dan jabatan. Jangan tulis kata sandi, PIN, atau token (USULAN).</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n"/>
+      <c r="D20" s="23" t="n"/>
+      <c r="E20" s="23" t="n"/>
     </row>
     <row r="21" ht="23.85" customHeight="1" s="12">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
@@ -744,69 +821,102 @@
           <t>Finance Lead meninjau isi berkas ini setiap tahun (USULAN).</t>
         </is>
       </c>
+      <c r="C21" s="23" t="n"/>
+      <c r="D21" s="23" t="n"/>
+      <c r="E21" s="23" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="12">
-      <c r="A22" s="18" t="n"/>
+      <c r="A22" s="19" t="n"/>
       <c r="B22" s="19" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" t="inlineStr">
+      <c r="C22" s="23" t="n"/>
+      <c r="D22" s="23" t="n"/>
+      <c r="E22" s="23" t="n"/>
+    </row>
+    <row r="23" ht="43.5" customHeight="1" s="12">
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>Finance Staff: peran pelaksana yang dijalankan pemegang jabatan Finance (JA-10) dan Accounting &amp; Tax (JA-11) (USULAN).</t>
         </is>
       </c>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
-      <c r="A24" s="17" t="n"/>
+      <c r="A24" s="25" t="n"/>
+      <c r="B24" s="23" t="n"/>
+      <c r="C24" s="23" t="n"/>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="12">
-      <c r="A25" s="20" t="n"/>
-      <c r="B25" s="18" t="n"/>
+      <c r="A25" s="26" t="n"/>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="23" t="n"/>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="23" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="12">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="18" t="n"/>
+      <c r="A26" s="26" t="n"/>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="12">
-      <c r="A27" s="20" t="n"/>
-      <c r="B27" s="18" t="n"/>
-    </row>
-    <row r="28"/>
-    <row r="29" ht="15" customHeight="1" s="12">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A27" s="26" t="n"/>
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="D27" s="23" t="n"/>
+      <c r="E27" s="23" t="n"/>
+    </row>
+    <row r="28" s="12">
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="23" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="12">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>Riwayat revisi</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="12">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="B29" s="23" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="D29" s="23" t="n"/>
+      <c r="E29" s="23" t="n"/>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="12">
+      <c r="A30" s="27" t="inlineStr">
         <is>
           <t>Revisi</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>Tanggal</t>
         </is>
       </c>
-      <c r="C30" s="21" t="inlineStr">
+      <c r="C30" s="27" t="inlineStr">
         <is>
           <t>Uraian perubahan</t>
         </is>
       </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="D30" s="27" t="inlineStr">
         <is>
           <t>Disusun</t>
         </is>
       </c>
-      <c r="E30" s="21" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>Disetujui</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="23.85" customHeight="1" s="12">
+    <row r="31" ht="30" customHeight="1" s="12">
       <c r="A31" s="16" t="inlineStr">
         <is>
           <t>00</t>
@@ -840,80 +950,95 @@
       <c r="D32" s="16" t="n"/>
       <c r="E32" s="16" t="n"/>
     </row>
-    <row r="33"/>
-    <row r="34" ht="15" customHeight="1" s="12">
-      <c r="A34" s="17" t="inlineStr">
+    <row r="33" s="12">
+      <c r="A33" s="23" t="n"/>
+      <c r="B33" s="23" t="n"/>
+      <c r="C33" s="23" t="n"/>
+      <c r="D33" s="23" t="n"/>
+      <c r="E33" s="23" t="n"/>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="12">
+      <c r="A34" s="25" t="inlineStr">
         <is>
           <t>Pengesahan</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="12">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="B34" s="23" t="n"/>
+      <c r="C34" s="23" t="n"/>
+      <c r="D34" s="23" t="n"/>
+      <c r="E34" s="23" t="n"/>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="12">
+      <c r="A35" s="27" t="inlineStr">
         <is>
           <t>Peran</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
+      <c r="B35" s="27" t="inlineStr">
         <is>
           <t>Nama dan jabatan</t>
         </is>
       </c>
-      <c r="C35" s="21" t="inlineStr">
+      <c r="C35" s="27" t="inlineStr">
         <is>
           <t>Tanda tangan</t>
         </is>
       </c>
-      <c r="D35" s="21" t="inlineStr">
+      <c r="D35" s="27" t="inlineStr">
         <is>
           <t>Tanggal</t>
         </is>
       </c>
+      <c r="E35" s="23" t="n"/>
     </row>
     <row r="36" ht="27.75" customHeight="1" s="12">
-      <c r="A36" s="22" t="inlineStr">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>Disusun oleh</t>
         </is>
       </c>
-      <c r="B36" s="22" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>Finance Staff</t>
         </is>
       </c>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
+      <c r="C36" s="16" t="n"/>
+      <c r="D36" s="16" t="n"/>
+      <c r="E36" s="23" t="n"/>
     </row>
     <row r="37" ht="27.75" customHeight="1" s="12">
-      <c r="A37" s="22" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Diperiksa oleh</t>
         </is>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Amirull Yusuf Zulkarnain / Direktur</t>
         </is>
       </c>
-      <c r="C37" s="22" t="n"/>
-      <c r="D37" s="22" t="n"/>
+      <c r="C37" s="16" t="n"/>
+      <c r="D37" s="16" t="n"/>
+      <c r="E37" s="23" t="n"/>
     </row>
     <row r="38" ht="27.75" customHeight="1" s="12">
-      <c r="A38" s="22" t="inlineStr">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>Disetujui oleh</t>
         </is>
       </c>
-      <c r="B38" s="22" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>Samuel Kristanto Utomo / President Director</t>
         </is>
       </c>
-      <c r="C38" s="22" t="n"/>
-      <c r="D38" s="22" t="n"/>
+      <c r="C38" s="16" t="n"/>
+      <c r="D38" s="16" t="n"/>
+      <c r="E38" s="23" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -921,17 +1046,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="27.88" customWidth="1" style="12" min="1" max="1"/>
     <col width="41.88" customWidth="1" style="12" min="2" max="2"/>
-    <col width="33" customWidth="1" style="12" min="4" max="4"/>
+    <col width="13" customWidth="1" style="12" min="3" max="3"/>
+    <col width="95" customWidth="1" style="12" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32.7" customHeight="1" s="12">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Document Name</t>
@@ -953,8 +1079,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="47.6" customHeight="1" s="12">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Worksheet PPh 21 Masa &amp; Tahunan</t>
         </is>
@@ -975,8 +1101,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="92.09999999999999" customHeight="1" s="12">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Tax Outstanding SINUX</t>
         </is>
@@ -990,7 +1116,7 @@
 4. PPh Badan</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>FAT</t>
         </is>
@@ -1001,7 +1127,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="62.4" customHeight="1" s="12">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>AR &amp; AP Aging</t>
@@ -1013,7 +1139,7 @@
 Dokumen akan diperbarui setiap tahun</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>FAT</t>
         </is>
@@ -1024,8 +1150,8 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="47.6" customHeight="1" s="12">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Fixed Asset</t>
         </is>
@@ -1035,7 +1161,7 @@
           <t>Dokumen list fixed asset lengkap dengan nama aset, nominal, tahun pembelian dan nilai buku terkini</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>FAT</t>
         </is>
@@ -1054,6 +1180,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1061,23 +1188,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="14.5" customWidth="1" style="12" min="1" max="1"/>
-    <col width="27.38" customWidth="1" style="12" min="2" max="2"/>
-    <col width="28.75" customWidth="1" style="12" min="3" max="3"/>
+    <col width="70" customWidth="1" style="12" min="2" max="2"/>
+    <col width="45" customWidth="1" style="12" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="17.9" customHeight="1" s="12">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Login Info</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
@@ -1088,8 +1215,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="17.9" customHeight="1" s="12">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Coretax</t>
         </is>
@@ -1105,8 +1232,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="107" customHeight="1" s="12">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>BCA Bank Access</t>
         </is>
@@ -1124,7 +1251,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="32.7" customHeight="1" s="12">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Artha Graha 
@@ -1142,33 +1269,33 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="10" t="n"/>
+    <row r="5" s="12">
+      <c r="A5" s="11" t="n"/>
       <c r="B5" s="11" t="n"/>
       <c r="C5" s="11" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="10" t="n"/>
+    <row r="6" s="12">
+      <c r="A6" s="11" t="n"/>
       <c r="B6" s="11" t="n"/>
       <c r="C6" s="11" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="n"/>
+    <row r="7" s="12">
+      <c r="A7" s="11" t="n"/>
       <c r="B7" s="11" t="n"/>
       <c r="C7" s="11" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="n"/>
+    <row r="8" s="12">
+      <c r="A8" s="11" t="n"/>
       <c r="B8" s="11" t="n"/>
       <c r="C8" s="11" t="n"/>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="n"/>
+    <row r="9" s="12">
+      <c r="A9" s="11" t="n"/>
       <c r="B9" s="11" t="n"/>
       <c r="C9" s="11" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="n"/>
+    <row r="10" s="12">
+      <c r="A10" s="11" t="n"/>
       <c r="B10" s="11" t="n"/>
       <c r="C10" s="11" t="n"/>
     </row>
@@ -1179,5 +1306,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
LEAD W11: verifikasi W10, koreksi cakupan 53 path di 25 dokumen, Master List dibangun ulang
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0159PhF1EfdAQgraQwR2djAZ
</commit_message>
<xml_diff>
--- a/out/03_FAT/SNX-FAT-FRM-02 Financial Information Access Authorization Records (Rev00 DRAFT).xlsx
+++ b/out/03_FAT/SNX-FAT-FRM-02 Financial Information Access Authorization Records (Rev00 DRAFT).xlsx
@@ -788,14 +788,14 @@
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>Isi sheet Platform Access dengan satu baris untuk setiap platform (USULAN).</t>
+          <t>Finance Staff mengisi sheet Platform Access dengan satu baris untuk setiap platform (USULAN).</t>
         </is>
       </c>
       <c r="C19" s="23" t="n"/>
       <c r="D19" s="23" t="n"/>
       <c r="E19" s="23" t="n"/>
     </row>
-    <row r="20" ht="30" customHeight="1" s="12">
+    <row r="20" ht="43.5" customHeight="1" s="12">
       <c r="A20" s="19" t="inlineStr">
         <is>
           <t>3.</t>
@@ -803,7 +803,7 @@
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>Tulis pemegang akses sebagai kelompok atau sebagai nama dan jabatan. Jangan tulis kata sandi, PIN, atau token (USULAN).</t>
+          <t>Finance Staff menulis pemegang akses sebagai kelompok atau sebagai nama dan jabatan, tanpa kata sandi, PIN, atau token (USULAN).</t>
         </is>
       </c>
       <c r="C20" s="23" t="n"/>

</xml_diff>